<commit_message>
Add Packing List feature and optimize Excel parsing
</commit_message>
<xml_diff>
--- a/public/templates/combination.xlsx
+++ b/public/templates/combination.xlsx
@@ -7,10 +7,10 @@
     <workbookView windowWidth="27947" windowHeight="12300"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="combination-5柜" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet1!$O$1:$O$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'combination-5柜'!$D$1:$D$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,21 +30,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="34">
   <si>
     <t>brutto</t>
-  </si>
-  <si>
-    <t>netto</t>
   </si>
   <si>
     <t>CNTR NO.</t>
   </si>
   <si>
-    <t>No. Of client</t>
+    <t>Block No.</t>
   </si>
   <si>
-    <t>Block No.</t>
+    <t>CLASS</t>
   </si>
   <si>
     <t>长</t>
@@ -62,16 +59,79 @@
     <t>Tons</t>
   </si>
   <si>
-    <t>CLASS</t>
+    <t>0208</t>
   </si>
   <si>
-    <t>UNIT PRICE</t>
+    <t>/25</t>
   </si>
   <si>
-    <t>说明：J列-Q列可有可无！</t>
+    <t>S III</t>
   </si>
   <si>
-    <t>说明：A列即柜号需要合并单元格</t>
+    <t>0206</t>
+  </si>
+  <si>
+    <t>S IV</t>
+  </si>
+  <si>
+    <t>0210</t>
+  </si>
+  <si>
+    <t>S II</t>
+  </si>
+  <si>
+    <t>0205</t>
+  </si>
+  <si>
+    <t>0209</t>
+  </si>
+  <si>
+    <t>0211</t>
+  </si>
+  <si>
+    <t>0255</t>
+  </si>
+  <si>
+    <t>0212</t>
+  </si>
+  <si>
+    <t>0250</t>
+  </si>
+  <si>
+    <t>0257</t>
+  </si>
+  <si>
+    <t>S I</t>
+  </si>
+  <si>
+    <t>0256</t>
+  </si>
+  <si>
+    <t>0214</t>
+  </si>
+  <si>
+    <t>0252</t>
+  </si>
+  <si>
+    <t>0207</t>
+  </si>
+  <si>
+    <t>0254</t>
+  </si>
+  <si>
+    <t>0251</t>
+  </si>
+  <si>
+    <t>0253</t>
+  </si>
+  <si>
+    <t>0259</t>
+  </si>
+  <si>
+    <t>0258</t>
+  </si>
+  <si>
+    <t>0213</t>
   </si>
 </sst>
 </file>
@@ -85,7 +145,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,16 +162,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="11.25"/>
+      <color rgb="FF1A2029"/>
+      <name val="PingFang SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11.25"/>
-      <color rgb="FF1A2029"/>
-      <name val="PingFang SC"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
@@ -265,12 +337,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -465,7 +543,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -510,6 +588,36 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -628,178 +736,215 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1150,121 +1295,2205 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:M140"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="1" max="15" width="9" style="1"/>
-    <col min="16" max="16" width="10.6666666666667" style="1" customWidth="1"/>
-    <col min="17" max="17" width="11.7777777777778" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="9" style="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="F1" s="2" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2" t="s">
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="4"/>
-    </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+    </row>
+    <row r="3" ht="15.6" spans="1:13">
+      <c r="A3" s="9">
+        <v>1</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="12">
+        <v>230</v>
+      </c>
+      <c r="F3" s="13">
+        <v>125</v>
+      </c>
+      <c r="G3" s="13">
+        <v>125</v>
+      </c>
+      <c r="H3" s="14">
+        <f>E3*F3*G3*0.000001</f>
+        <v>3.59375</v>
+      </c>
+      <c r="I3" s="15">
+        <v>7.95</v>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" ht="15.6" spans="1:13">
+      <c r="A4" s="9"/>
+      <c r="B4" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="12">
+        <v>250</v>
+      </c>
+      <c r="F4" s="13">
+        <v>80</v>
+      </c>
+      <c r="G4" s="13">
+        <v>83</v>
+      </c>
+      <c r="H4" s="14">
+        <f>E4*F4*G4*0.000001</f>
+        <v>1.66</v>
+      </c>
+      <c r="I4" s="15">
+        <v>4.35</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+    </row>
+    <row r="5" ht="15.6" spans="1:13">
+      <c r="A5" s="9"/>
+      <c r="B5" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="17">
+        <v>210</v>
+      </c>
+      <c r="F5" s="18">
+        <v>150</v>
+      </c>
+      <c r="G5" s="18">
+        <v>120</v>
+      </c>
+      <c r="H5" s="19">
+        <f>E5*F5*G5*0.000001</f>
+        <v>3.78</v>
+      </c>
+      <c r="I5" s="20">
+        <v>9.61</v>
+      </c>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+    </row>
+    <row r="6" ht="15.6" spans="1:13">
+      <c r="A6" s="9"/>
+      <c r="B6" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="17">
+        <v>214</v>
+      </c>
+      <c r="F6" s="18">
+        <v>124</v>
+      </c>
+      <c r="G6" s="18">
+        <v>55</v>
+      </c>
+      <c r="H6" s="19">
+        <f>E6*F6*G6*0.000001</f>
+        <v>1.45948</v>
+      </c>
+      <c r="I6" s="20">
+        <v>3.35</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1">
+        <f>+E4+F5+F6</f>
+        <v>524</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="22">
+        <f>SUM(I3:I6)</f>
+        <v>25.26</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" ht="15.6" spans="1:13">
+      <c r="A9" s="9">
+        <v>2</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="12">
+        <v>230</v>
+      </c>
+      <c r="F9" s="13">
+        <v>90</v>
+      </c>
+      <c r="G9" s="13">
+        <v>125</v>
+      </c>
+      <c r="H9" s="14">
+        <f>E9*F9*G9*0.000001</f>
+        <v>2.5875</v>
+      </c>
+      <c r="I9" s="15">
+        <v>6.42</v>
+      </c>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" ht="15.6" spans="1:13">
+      <c r="A10" s="9"/>
+      <c r="B10" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="12">
+        <v>250</v>
+      </c>
+      <c r="F10" s="13">
+        <v>150</v>
+      </c>
+      <c r="G10" s="13">
+        <v>115</v>
+      </c>
+      <c r="H10" s="14">
+        <f>E10*F10*G10*0.000001</f>
+        <v>4.3125</v>
+      </c>
+      <c r="I10" s="15">
+        <v>10.67</v>
+      </c>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" ht="15.6" spans="1:13">
+      <c r="A11" s="9"/>
+      <c r="B11" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="17">
+        <v>210</v>
+      </c>
+      <c r="F11" s="18">
+        <v>120</v>
+      </c>
+      <c r="G11" s="18">
+        <v>75</v>
+      </c>
+      <c r="H11" s="19">
+        <f>E11*F11*G11*0.000001</f>
+        <v>1.89</v>
+      </c>
+      <c r="I11" s="20">
+        <v>4.45</v>
+      </c>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" ht="15.6" spans="1:13">
+      <c r="A12" s="9"/>
+      <c r="B12" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="17">
+        <v>170</v>
+      </c>
+      <c r="F12" s="18">
+        <v>110</v>
+      </c>
+      <c r="G12" s="18">
+        <v>70</v>
+      </c>
+      <c r="H12" s="19">
+        <f>E12*F12*G12*0.000001</f>
+        <v>1.309</v>
+      </c>
+      <c r="I12" s="20">
+        <v>3.47</v>
+      </c>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1">
+        <f>+E10+F11+F12</f>
+        <v>480</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="22">
+        <f>SUM(I9:I12)</f>
+        <v>25.01</v>
+      </c>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+    </row>
+    <row r="15" ht="15.6" spans="1:13">
+      <c r="A15" s="9">
+        <v>3</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="12">
+        <v>273</v>
+      </c>
+      <c r="F15" s="13">
+        <v>180</v>
+      </c>
+      <c r="G15" s="13">
+        <v>85</v>
+      </c>
+      <c r="H15" s="14">
+        <f>E15*F15*G15*0.000001</f>
+        <v>4.1769</v>
+      </c>
+      <c r="I15" s="15">
+        <v>9.85</v>
+      </c>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" ht="15.6" spans="1:13">
+      <c r="A16" s="9"/>
+      <c r="B16" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="12">
+        <v>233</v>
+      </c>
+      <c r="F16" s="13">
+        <v>122</v>
+      </c>
+      <c r="G16" s="13">
+        <v>78</v>
+      </c>
+      <c r="H16" s="14">
+        <f>E16*F16*G16*0.000001</f>
+        <v>2.217228</v>
+      </c>
+      <c r="I16" s="15">
+        <v>5.31</v>
+      </c>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" ht="15.6" spans="1:13">
+      <c r="A17" s="9"/>
+      <c r="B17" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="17">
+        <v>210</v>
+      </c>
+      <c r="F17" s="18">
+        <v>195</v>
+      </c>
+      <c r="G17" s="18">
+        <v>70</v>
+      </c>
+      <c r="H17" s="19">
+        <f>E17*F17*G17*0.000001</f>
+        <v>2.8665</v>
+      </c>
+      <c r="I17" s="20">
+        <v>7.11</v>
+      </c>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" ht="15.6" spans="1:13">
+      <c r="A18" s="9"/>
+      <c r="B18" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="17">
+        <v>155</v>
+      </c>
+      <c r="F18" s="18">
+        <v>120</v>
+      </c>
+      <c r="G18" s="18">
+        <v>60</v>
+      </c>
+      <c r="H18" s="19">
+        <f>E18*F18*G18*0.000001</f>
+        <v>1.116</v>
+      </c>
+      <c r="I18" s="20">
+        <v>2.88</v>
+      </c>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1">
+        <f>+E15+F17+G18</f>
+        <v>528</v>
+      </c>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="22">
+        <f>SUM(I15:I18)</f>
+        <v>25.15</v>
+      </c>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+    </row>
+    <row r="21" ht="15.6" spans="1:13">
+      <c r="A21" s="9">
+        <v>4</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="12">
+        <v>290</v>
+      </c>
+      <c r="F21" s="13">
+        <v>160</v>
+      </c>
+      <c r="G21" s="13">
+        <v>63</v>
+      </c>
+      <c r="H21" s="14">
+        <f>E21*F21*G21*0.000001</f>
+        <v>2.9232</v>
+      </c>
+      <c r="I21" s="15">
+        <v>7.28</v>
+      </c>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" ht="15.6" spans="1:13">
+      <c r="A22" s="9"/>
+      <c r="B22" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="12">
+        <v>190</v>
+      </c>
+      <c r="F22" s="13">
+        <v>110</v>
+      </c>
+      <c r="G22" s="13">
+        <v>95</v>
+      </c>
+      <c r="H22" s="14">
+        <f>E22*F22*G22*0.000001</f>
+        <v>1.9855</v>
+      </c>
+      <c r="I22" s="15">
+        <v>5.09</v>
+      </c>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+    </row>
+    <row r="23" ht="15.6" spans="1:13">
+      <c r="A23" s="9"/>
+      <c r="B23" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="17">
+        <v>175</v>
+      </c>
+      <c r="F23" s="18">
+        <v>140</v>
+      </c>
+      <c r="G23" s="18">
+        <v>110</v>
+      </c>
+      <c r="H23" s="19">
+        <f>E23*F23*G23*0.000001</f>
+        <v>2.695</v>
+      </c>
+      <c r="I23" s="20">
+        <v>6.79</v>
+      </c>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+    </row>
+    <row r="24" ht="15.6" spans="1:13">
+      <c r="A24" s="9"/>
+      <c r="B24" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="17">
+        <v>190</v>
+      </c>
+      <c r="F24" s="18">
+        <v>140</v>
+      </c>
+      <c r="G24" s="18">
+        <v>100</v>
+      </c>
+      <c r="H24" s="19">
+        <f>E24*F24*G24*0.000001</f>
+        <v>2.66</v>
+      </c>
+      <c r="I24" s="20">
+        <v>6.35</v>
+      </c>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1">
+        <f>+E21+F23+F24</f>
+        <v>570</v>
+      </c>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="22">
+        <f>SUM(I21:I24)</f>
+        <v>25.51</v>
+      </c>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+    </row>
+    <row r="27" ht="15.6" spans="1:13">
+      <c r="A27" s="9">
         <v>5</v>
       </c>
-      <c r="K2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="O2" s="7" t="s">
+      <c r="B27" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="D27" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="12">
+        <v>225</v>
+      </c>
+      <c r="F27" s="13">
+        <v>130</v>
+      </c>
+      <c r="G27" s="13">
+        <v>110</v>
+      </c>
+      <c r="H27" s="14">
+        <f>E27*F27*G27*0.000001</f>
+        <v>3.2175</v>
+      </c>
+      <c r="I27" s="15">
+        <v>8.07</v>
+      </c>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+    </row>
+    <row r="28" ht="15.6" spans="1:13">
+      <c r="A28" s="9"/>
+      <c r="B28" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="12">
+        <v>252</v>
+      </c>
+      <c r="F28" s="13">
+        <v>105</v>
+      </c>
+      <c r="G28" s="13">
+        <v>195</v>
+      </c>
+      <c r="H28" s="14">
+        <f>E28*F28*G28*0.000001</f>
+        <v>5.1597</v>
+      </c>
+      <c r="I28" s="15">
+        <v>12.48</v>
+      </c>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+    </row>
+    <row r="29" ht="15.6" spans="1:13">
+      <c r="A29" s="9"/>
+      <c r="B29" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="17">
+        <v>173</v>
+      </c>
+      <c r="F29" s="18">
+        <v>95</v>
+      </c>
+      <c r="G29" s="18">
+        <v>65</v>
+      </c>
+      <c r="H29" s="19">
+        <f>E29*F29*G29*0.000001</f>
+        <v>1.068275</v>
+      </c>
+      <c r="I29" s="20">
+        <v>2.61</v>
+      </c>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+    </row>
+    <row r="30" ht="15.6" spans="1:13">
+      <c r="A30" s="9"/>
+      <c r="B30" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="B6" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-    </row>
-    <row r="7" spans="1:16">
-      <c r="B7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-    </row>
-    <row r="8" ht="15.6" spans="1:16">
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="13"/>
-    </row>
-    <row r="18" spans="2:8">
-      <c r="B18" s="14"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="E30" s="17">
+        <v>200</v>
+      </c>
+      <c r="F30" s="18">
+        <v>100</v>
+      </c>
+      <c r="G30" s="18">
+        <v>50</v>
+      </c>
+      <c r="H30" s="19">
+        <f>E30*F30*G30*0.000001</f>
+        <v>1</v>
+      </c>
+      <c r="I30" s="20">
+        <v>2.6</v>
+      </c>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="1">
+        <f>+E28+F30+F29</f>
+        <v>447</v>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="21">
+        <f>SUM(I27:I30)</f>
+        <v>25.76</v>
+      </c>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+    </row>
+    <row r="35" ht="15.6" spans="1:13">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="25">
+        <f>SUM(H3:H29)</f>
+        <v>50.678033</v>
+      </c>
+      <c r="I35" s="25">
+        <v>126.69</v>
+      </c>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="1"/>
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="1"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="26"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27"/>
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+    </row>
+    <row r="48" spans="1:13">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="1"/>
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+    </row>
+    <row r="49" spans="1:13">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="1"/>
+      <c r="J49" s="1"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+    </row>
+    <row r="50" spans="1:13">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+    </row>
+    <row r="51" spans="1:13">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="1"/>
+      <c r="J51" s="1"/>
+      <c r="K51" s="1"/>
+      <c r="L51" s="1"/>
+      <c r="M51" s="1"/>
+    </row>
+    <row r="52" spans="1:13">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+    </row>
+    <row r="53" spans="1:13">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+    </row>
+    <row r="54" spans="1:13">
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+    </row>
+    <row r="55" spans="1:13">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+    </row>
+    <row r="56" spans="1:13">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+    </row>
+    <row r="57" spans="1:13">
+      <c r="A57" s="1"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+    </row>
+    <row r="58" spans="1:13">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+    </row>
+    <row r="59" spans="1:13">
+      <c r="A59" s="1"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
+      <c r="J59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+    </row>
+    <row r="60" spans="1:13">
+      <c r="A60" s="1"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+    </row>
+    <row r="61" spans="1:13">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="1"/>
+      <c r="J61" s="1"/>
+      <c r="K61" s="1"/>
+      <c r="L61" s="1"/>
+      <c r="M61" s="1"/>
+    </row>
+    <row r="62" spans="1:13">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="1"/>
+      <c r="J62" s="1"/>
+      <c r="K62" s="1"/>
+      <c r="L62" s="1"/>
+      <c r="M62" s="1"/>
+    </row>
+    <row r="63" spans="1:13">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="1"/>
+      <c r="J63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="1"/>
+      <c r="M63" s="1"/>
+    </row>
+    <row r="64" spans="1:13">
+      <c r="A64" s="1"/>
+      <c r="B64" s="1"/>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="1"/>
+      <c r="J64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="L64" s="1"/>
+      <c r="M64" s="1"/>
+    </row>
+    <row r="65" spans="1:13">
+      <c r="A65" s="1"/>
+      <c r="B65" s="1"/>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="I65" s="1"/>
+      <c r="J65" s="1"/>
+      <c r="K65" s="1"/>
+      <c r="L65" s="1"/>
+      <c r="M65" s="1"/>
+    </row>
+    <row r="66" spans="1:13">
+      <c r="A66" s="1"/>
+      <c r="B66" s="1"/>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="1"/>
+      <c r="M66" s="1"/>
+    </row>
+    <row r="67" spans="1:13">
+      <c r="A67" s="1"/>
+      <c r="B67" s="1"/>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+      <c r="I67" s="1"/>
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="1"/>
+      <c r="M67" s="1"/>
+    </row>
+    <row r="68" spans="1:13">
+      <c r="A68" s="1"/>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="1"/>
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="L68" s="1"/>
+      <c r="M68" s="1"/>
+    </row>
+    <row r="69" spans="1:13">
+      <c r="A69" s="1"/>
+      <c r="B69" s="1"/>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="1"/>
+      <c r="J69" s="1"/>
+      <c r="K69" s="1"/>
+      <c r="L69" s="1"/>
+      <c r="M69" s="1"/>
+    </row>
+    <row r="70" spans="1:13">
+      <c r="A70" s="1"/>
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="1"/>
+      <c r="J70" s="1"/>
+      <c r="K70" s="1"/>
+      <c r="L70" s="1"/>
+      <c r="M70" s="1"/>
+    </row>
+    <row r="71" spans="1:13">
+      <c r="A71" s="1"/>
+      <c r="B71" s="1"/>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
+    </row>
+    <row r="72" spans="1:13">
+      <c r="A72" s="1"/>
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="1"/>
+      <c r="H72" s="1"/>
+      <c r="I72" s="1"/>
+      <c r="J72" s="1"/>
+      <c r="K72" s="1"/>
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
+    </row>
+    <row r="73" spans="1:13">
+      <c r="A73" s="1"/>
+      <c r="B73" s="1"/>
+      <c r="C73" s="1"/>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1"/>
+      <c r="G73" s="1"/>
+      <c r="H73" s="1"/>
+      <c r="I73" s="1"/>
+    </row>
+    <row r="74" spans="1:13">
+      <c r="A74" s="1"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
+      <c r="I74" s="1"/>
+    </row>
+    <row r="75" spans="1:13">
+      <c r="A75" s="1"/>
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+      <c r="I75" s="1"/>
+    </row>
+    <row r="76" spans="1:13">
+      <c r="A76" s="1"/>
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+      <c r="I76" s="1"/>
+    </row>
+    <row r="77" spans="1:13">
+      <c r="A77" s="1"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
+      <c r="I77" s="1"/>
+    </row>
+    <row r="78" spans="1:13">
+      <c r="A78" s="1"/>
+      <c r="B78" s="1"/>
+      <c r="C78" s="1"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="1"/>
+      <c r="H78" s="1"/>
+      <c r="I78" s="1"/>
+    </row>
+    <row r="79" spans="1:13">
+      <c r="A79" s="1"/>
+      <c r="B79" s="1"/>
+      <c r="C79" s="1"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1"/>
+      <c r="G79" s="1"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="1"/>
+    </row>
+    <row r="80" spans="1:13">
+      <c r="A80" s="1"/>
+      <c r="B80" s="1"/>
+      <c r="C80" s="1"/>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+      <c r="F80" s="1"/>
+      <c r="G80" s="1"/>
+      <c r="H80" s="1"/>
+      <c r="I80" s="1"/>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" s="1"/>
+      <c r="B81" s="1"/>
+      <c r="C81" s="1"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="1"/>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" s="1"/>
+      <c r="B82" s="1"/>
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+      <c r="F82" s="1"/>
+      <c r="G82" s="1"/>
+      <c r="H82" s="1"/>
+      <c r="I82" s="1"/>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" s="1"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+      <c r="I83" s="1"/>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" s="1"/>
+      <c r="B84" s="1"/>
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1"/>
+      <c r="G84" s="1"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="1"/>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" s="1"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="1"/>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" s="1"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+      <c r="I87" s="1"/>
+    </row>
+    <row r="88" spans="1:9">
+      <c r="A88" s="1"/>
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="1"/>
+      <c r="I88" s="1"/>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" s="1"/>
+      <c r="B89" s="1"/>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="1"/>
+      <c r="I89" s="1"/>
+    </row>
+    <row r="90" spans="1:9">
+      <c r="A90" s="1"/>
+      <c r="B90" s="1"/>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
+    </row>
+    <row r="91" spans="1:9">
+      <c r="A91" s="1"/>
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
+    </row>
+    <row r="92" spans="1:9">
+      <c r="A92" s="1"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+    </row>
+    <row r="93" spans="1:9">
+      <c r="A93" s="1"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
+    </row>
+    <row r="94" spans="1:9">
+      <c r="A94" s="1"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
+    </row>
+    <row r="95" spans="1:9">
+      <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="1"/>
+      <c r="I95" s="1"/>
+    </row>
+    <row r="96" spans="1:9">
+      <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
+    </row>
+    <row r="97" spans="1:9">
+      <c r="A97" s="1"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1"/>
+      <c r="G97" s="1"/>
+      <c r="H97" s="1"/>
+      <c r="I97" s="1"/>
+    </row>
+    <row r="98" spans="1:9">
+      <c r="A98" s="1"/>
+      <c r="B98" s="1"/>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="1"/>
+      <c r="I98" s="1"/>
+    </row>
+    <row r="99" spans="1:9">
+      <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="1"/>
+      <c r="I99" s="1"/>
+    </row>
+    <row r="100" spans="1:9">
+      <c r="A100" s="1"/>
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="1"/>
+      <c r="I100" s="1"/>
+    </row>
+    <row r="101" spans="1:9">
+      <c r="A101" s="1"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="1"/>
+      <c r="I101" s="1"/>
+    </row>
+    <row r="102" spans="1:9">
+      <c r="A102" s="1"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="1"/>
+      <c r="I102" s="1"/>
+    </row>
+    <row r="103" spans="1:9">
+      <c r="A103" s="1"/>
+      <c r="B103" s="1"/>
+      <c r="C103" s="1"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="1"/>
+      <c r="I103" s="1"/>
+    </row>
+    <row r="104" spans="1:9">
+      <c r="A104" s="1"/>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="1"/>
+      <c r="I104" s="1"/>
+    </row>
+    <row r="105" spans="1:9">
+      <c r="A105" s="1"/>
+      <c r="B105" s="1"/>
+      <c r="C105" s="1"/>
+      <c r="D105" s="1"/>
+      <c r="E105" s="1"/>
+      <c r="F105" s="1"/>
+      <c r="G105" s="1"/>
+      <c r="H105" s="1"/>
+      <c r="I105" s="1"/>
+    </row>
+    <row r="106" spans="1:9">
+      <c r="A106" s="1"/>
+      <c r="B106" s="1"/>
+      <c r="C106" s="1"/>
+      <c r="D106" s="1"/>
+      <c r="E106" s="1"/>
+      <c r="F106" s="1"/>
+      <c r="G106" s="1"/>
+      <c r="H106" s="1"/>
+      <c r="I106" s="1"/>
+    </row>
+    <row r="107" spans="1:9">
+      <c r="A107" s="1"/>
+      <c r="B107" s="1"/>
+      <c r="C107" s="1"/>
+      <c r="D107" s="1"/>
+      <c r="E107" s="1"/>
+      <c r="F107" s="1"/>
+      <c r="G107" s="1"/>
+      <c r="H107" s="1"/>
+      <c r="I107" s="1"/>
+    </row>
+    <row r="108" spans="1:9">
+      <c r="A108" s="1"/>
+      <c r="B108" s="1"/>
+      <c r="C108" s="1"/>
+      <c r="D108" s="1"/>
+      <c r="E108" s="1"/>
+      <c r="F108" s="1"/>
+      <c r="G108" s="1"/>
+      <c r="H108" s="1"/>
+      <c r="I108" s="1"/>
+    </row>
+    <row r="109" spans="1:9">
+      <c r="A109" s="1"/>
+      <c r="B109" s="1"/>
+      <c r="C109" s="1"/>
+      <c r="D109" s="1"/>
+      <c r="E109" s="1"/>
+      <c r="F109" s="1"/>
+      <c r="G109" s="1"/>
+      <c r="H109" s="1"/>
+      <c r="I109" s="1"/>
+    </row>
+    <row r="110" spans="1:9">
+      <c r="A110" s="1"/>
+      <c r="B110" s="1"/>
+      <c r="C110" s="1"/>
+      <c r="D110" s="1"/>
+      <c r="E110" s="1"/>
+      <c r="F110" s="1"/>
+      <c r="G110" s="1"/>
+      <c r="H110" s="1"/>
+      <c r="I110" s="1"/>
+    </row>
+    <row r="111" spans="1:9">
+      <c r="A111" s="1"/>
+      <c r="B111" s="1"/>
+      <c r="C111" s="1"/>
+      <c r="D111" s="1"/>
+      <c r="E111" s="1"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="1"/>
+      <c r="H111" s="1"/>
+      <c r="I111" s="1"/>
+    </row>
+    <row r="112" spans="1:9">
+      <c r="A112" s="1"/>
+      <c r="B112" s="1"/>
+      <c r="C112" s="1"/>
+      <c r="D112" s="1"/>
+      <c r="E112" s="1"/>
+      <c r="F112" s="1"/>
+      <c r="G112" s="1"/>
+      <c r="H112" s="1"/>
+      <c r="I112" s="1"/>
+    </row>
+    <row r="113" spans="1:9">
+      <c r="A113" s="1"/>
+      <c r="B113" s="1"/>
+      <c r="C113" s="1"/>
+      <c r="D113" s="1"/>
+      <c r="E113" s="1"/>
+      <c r="F113" s="1"/>
+      <c r="G113" s="1"/>
+      <c r="H113" s="1"/>
+      <c r="I113" s="1"/>
+    </row>
+    <row r="114" spans="1:9">
+      <c r="A114" s="1"/>
+      <c r="B114" s="1"/>
+      <c r="C114" s="1"/>
+      <c r="D114" s="1"/>
+      <c r="E114" s="1"/>
+      <c r="F114" s="1"/>
+      <c r="G114" s="1"/>
+      <c r="H114" s="1"/>
+      <c r="I114" s="1"/>
+    </row>
+    <row r="115" spans="1:9">
+      <c r="A115" s="1"/>
+      <c r="B115" s="1"/>
+      <c r="C115" s="1"/>
+      <c r="D115" s="1"/>
+      <c r="E115" s="1"/>
+      <c r="F115" s="1"/>
+      <c r="G115" s="1"/>
+      <c r="H115" s="1"/>
+      <c r="I115" s="1"/>
+    </row>
+    <row r="116" spans="1:9">
+      <c r="A116" s="1"/>
+      <c r="B116" s="1"/>
+      <c r="C116" s="1"/>
+      <c r="D116" s="1"/>
+      <c r="E116" s="1"/>
+      <c r="F116" s="1"/>
+      <c r="G116" s="1"/>
+      <c r="H116" s="1"/>
+      <c r="I116" s="1"/>
+    </row>
+    <row r="117" spans="1:9">
+      <c r="A117" s="1"/>
+      <c r="B117" s="1"/>
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+      <c r="F117" s="1"/>
+      <c r="G117" s="1"/>
+      <c r="H117" s="1"/>
+      <c r="I117" s="1"/>
+    </row>
+    <row r="118" spans="1:9">
+      <c r="A118" s="1"/>
+      <c r="B118" s="1"/>
+      <c r="C118" s="1"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+      <c r="F118" s="1"/>
+      <c r="G118" s="1"/>
+      <c r="H118" s="1"/>
+      <c r="I118" s="1"/>
+    </row>
+    <row r="119" spans="1:9">
+      <c r="A119" s="1"/>
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+      <c r="D119" s="1"/>
+      <c r="E119" s="1"/>
+      <c r="F119" s="1"/>
+      <c r="G119" s="1"/>
+      <c r="H119" s="1"/>
+      <c r="I119" s="1"/>
+    </row>
+    <row r="120" spans="1:9">
+      <c r="A120" s="1"/>
+      <c r="B120" s="1"/>
+      <c r="C120" s="1"/>
+      <c r="D120" s="1"/>
+      <c r="E120" s="1"/>
+      <c r="F120" s="1"/>
+      <c r="G120" s="1"/>
+      <c r="H120" s="1"/>
+      <c r="I120" s="1"/>
+    </row>
+    <row r="121" spans="1:9">
+      <c r="A121" s="1"/>
+      <c r="B121" s="1"/>
+      <c r="C121" s="1"/>
+      <c r="D121" s="1"/>
+      <c r="E121" s="1"/>
+      <c r="F121" s="1"/>
+      <c r="G121" s="1"/>
+      <c r="H121" s="1"/>
+      <c r="I121" s="1"/>
+    </row>
+    <row r="122" spans="1:9">
+      <c r="A122" s="1"/>
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="1"/>
+      <c r="E122" s="1"/>
+      <c r="F122" s="1"/>
+      <c r="G122" s="1"/>
+      <c r="H122" s="1"/>
+      <c r="I122" s="1"/>
+    </row>
+    <row r="123" spans="1:9">
+      <c r="A123" s="1"/>
+      <c r="B123" s="1"/>
+      <c r="C123" s="1"/>
+      <c r="D123" s="1"/>
+      <c r="E123" s="1"/>
+      <c r="F123" s="1"/>
+      <c r="G123" s="1"/>
+      <c r="H123" s="1"/>
+      <c r="I123" s="1"/>
+    </row>
+    <row r="124" spans="1:9">
+      <c r="A124" s="1"/>
+      <c r="B124" s="1"/>
+      <c r="C124" s="1"/>
+      <c r="D124" s="1"/>
+      <c r="E124" s="1"/>
+      <c r="F124" s="1"/>
+      <c r="G124" s="1"/>
+      <c r="H124" s="1"/>
+      <c r="I124" s="1"/>
+    </row>
+    <row r="125" spans="1:9">
+      <c r="A125" s="1"/>
+      <c r="B125" s="1"/>
+      <c r="C125" s="1"/>
+      <c r="D125" s="1"/>
+      <c r="E125" s="1"/>
+      <c r="F125" s="1"/>
+      <c r="G125" s="1"/>
+      <c r="H125" s="1"/>
+      <c r="I125" s="1"/>
+    </row>
+    <row r="126" spans="1:9">
+      <c r="A126" s="1"/>
+      <c r="B126" s="1"/>
+      <c r="C126" s="1"/>
+      <c r="D126" s="1"/>
+      <c r="E126" s="1"/>
+      <c r="F126" s="1"/>
+      <c r="G126" s="1"/>
+      <c r="H126" s="1"/>
+      <c r="I126" s="1"/>
+    </row>
+    <row r="127" spans="1:9">
+      <c r="A127" s="1"/>
+      <c r="B127" s="1"/>
+      <c r="C127" s="1"/>
+      <c r="D127" s="1"/>
+      <c r="E127" s="1"/>
+      <c r="F127" s="1"/>
+      <c r="G127" s="1"/>
+      <c r="H127" s="1"/>
+      <c r="I127" s="1"/>
+    </row>
+    <row r="128" spans="1:9">
+      <c r="A128" s="1"/>
+      <c r="B128" s="1"/>
+      <c r="C128" s="1"/>
+      <c r="D128" s="1"/>
+      <c r="E128" s="1"/>
+      <c r="F128" s="1"/>
+      <c r="G128" s="1"/>
+      <c r="H128" s="1"/>
+      <c r="I128" s="1"/>
+    </row>
+    <row r="129" spans="1:9">
+      <c r="A129" s="1"/>
+      <c r="B129" s="1"/>
+      <c r="C129" s="1"/>
+      <c r="D129" s="1"/>
+      <c r="E129" s="1"/>
+      <c r="F129" s="1"/>
+      <c r="G129" s="1"/>
+      <c r="H129" s="1"/>
+      <c r="I129" s="1"/>
+    </row>
+    <row r="130" spans="1:9">
+      <c r="A130" s="1"/>
+      <c r="B130" s="1"/>
+      <c r="C130" s="1"/>
+      <c r="D130" s="1"/>
+      <c r="E130" s="1"/>
+      <c r="F130" s="1"/>
+      <c r="G130" s="1"/>
+      <c r="H130" s="1"/>
+      <c r="I130" s="1"/>
+    </row>
+    <row r="131" spans="1:9">
+      <c r="A131" s="1"/>
+      <c r="B131" s="1"/>
+      <c r="C131" s="1"/>
+      <c r="D131" s="1"/>
+      <c r="E131" s="1"/>
+      <c r="F131" s="1"/>
+      <c r="G131" s="1"/>
+      <c r="H131" s="1"/>
+      <c r="I131" s="1"/>
+    </row>
+    <row r="132" spans="1:9">
+      <c r="A132" s="1"/>
+      <c r="B132" s="1"/>
+      <c r="C132" s="1"/>
+      <c r="D132" s="1"/>
+      <c r="E132" s="1"/>
+      <c r="F132" s="1"/>
+      <c r="G132" s="1"/>
+      <c r="H132" s="1"/>
+      <c r="I132" s="1"/>
+    </row>
+    <row r="133" spans="1:9">
+      <c r="A133" s="1"/>
+      <c r="B133" s="1"/>
+      <c r="C133" s="1"/>
+      <c r="D133" s="1"/>
+      <c r="E133" s="1"/>
+      <c r="F133" s="1"/>
+      <c r="G133" s="1"/>
+      <c r="H133" s="1"/>
+      <c r="I133" s="1"/>
+    </row>
+    <row r="134" spans="1:9">
+      <c r="A134" s="1"/>
+      <c r="B134" s="1"/>
+      <c r="C134" s="1"/>
+      <c r="D134" s="1"/>
+      <c r="E134" s="1"/>
+      <c r="F134" s="1"/>
+      <c r="G134" s="1"/>
+      <c r="H134" s="1"/>
+      <c r="I134" s="1"/>
+    </row>
+    <row r="135" spans="1:9">
+      <c r="A135" s="1"/>
+      <c r="B135" s="1"/>
+      <c r="C135" s="1"/>
+      <c r="D135" s="1"/>
+      <c r="E135" s="1"/>
+      <c r="F135" s="1"/>
+      <c r="G135" s="1"/>
+      <c r="H135" s="1"/>
+      <c r="I135" s="1"/>
+    </row>
+    <row r="136" spans="1:9">
+      <c r="A136" s="1"/>
+      <c r="B136" s="1"/>
+      <c r="C136" s="1"/>
+      <c r="D136" s="1"/>
+      <c r="E136" s="1"/>
+      <c r="F136" s="1"/>
+      <c r="G136" s="1"/>
+      <c r="H136" s="1"/>
+      <c r="I136" s="1"/>
+    </row>
+    <row r="137" spans="1:9">
+      <c r="A137" s="1"/>
+      <c r="B137" s="1"/>
+      <c r="C137" s="1"/>
+      <c r="D137" s="1"/>
+      <c r="E137" s="1"/>
+      <c r="F137" s="1"/>
+      <c r="G137" s="1"/>
+      <c r="H137" s="1"/>
+      <c r="I137" s="1"/>
+    </row>
+    <row r="138" spans="1:9">
+      <c r="A138" s="1"/>
+      <c r="B138" s="1"/>
+      <c r="C138" s="1"/>
+      <c r="D138" s="1"/>
+      <c r="E138" s="1"/>
+      <c r="F138" s="1"/>
+      <c r="G138" s="1"/>
+      <c r="H138" s="1"/>
+      <c r="I138" s="1"/>
+    </row>
+    <row r="139" spans="1:9">
+      <c r="A139" s="1"/>
+      <c r="B139" s="1"/>
+      <c r="C139" s="1"/>
+      <c r="D139" s="1"/>
+      <c r="E139" s="1"/>
+      <c r="F139" s="1"/>
+      <c r="G139" s="1"/>
+      <c r="H139" s="1"/>
+      <c r="I139" s="1"/>
+    </row>
+    <row r="140" spans="1:9">
+      <c r="A140" s="1"/>
+      <c r="B140" s="1"/>
+      <c r="C140" s="1"/>
+      <c r="D140" s="1"/>
+      <c r="E140" s="1"/>
+      <c r="F140" s="1"/>
+      <c r="G140" s="1"/>
+      <c r="H140" s="1"/>
+      <c r="I140" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:N1"/>
+  <mergeCells count="7">
+    <mergeCell ref="E1:H1"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A27:A30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>